<commit_message>
Integrate live official IMF FX Reserves scraper (RXF11FX_REVS) and synchronize database and frontend dataset
</commit_message>
<xml_diff>
--- a/VERIFIED_INDICATORS_EXPORT.xlsx
+++ b/VERIFIED_INDICATORS_EXPORT.xlsx
@@ -2240,7 +2240,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE9"/>
+  <dimension ref="A1:DA9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2251,280 +2251,520 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>2018-01-01</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>2018-02-01</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>2018-03-01</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>2018-04-01</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>2018-05-01</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>2018-06-01</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>2018-07-01</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>2018-08-01</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>2018-09-01</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>2018-10-01</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>2018-11-01</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>2018-12-01</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>2019-01-01</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>2019-02-01</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>2019-03-01</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>2019-04-01</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>2019-05-01</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>2019-06-01</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>2019-07-01</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>2019-08-01</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>2019-09-01</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>2019-10-01</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>2019-11-01</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>2019-12-01</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>2020-02-01</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>2020-03-01</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>2020-04-01</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>2020-05-01</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>2020-06-01</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>2020-07-01</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>2020-08-01</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>2020-09-01</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>2020-10-01</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>2020-11-01</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>2020-12-01</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>2021-01-01</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>2021-02-01</t>
+        </is>
+      </c>
+      <c r="AN1" t="inlineStr">
+        <is>
+          <t>2021-03-01</t>
+        </is>
+      </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>2021-04-01</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>2021-05-01</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>2021-06-01</t>
+        </is>
+      </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>2021-07-01</t>
+        </is>
+      </c>
+      <c r="AS1" t="inlineStr">
+        <is>
+          <t>2021-08-01</t>
+        </is>
+      </c>
+      <c r="AT1" t="inlineStr">
+        <is>
+          <t>2021-09-01</t>
+        </is>
+      </c>
+      <c r="AU1" t="inlineStr">
+        <is>
+          <t>2021-10-01</t>
+        </is>
+      </c>
+      <c r="AV1" t="inlineStr">
+        <is>
+          <t>2021-11-01</t>
+        </is>
+      </c>
+      <c r="AW1" t="inlineStr">
+        <is>
+          <t>2021-12-01</t>
+        </is>
+      </c>
+      <c r="AX1" t="inlineStr">
+        <is>
           <t>2022-01-01</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>2022-02-01</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>2022-03-01</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>2022-04-01</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
         <is>
           <t>2022-05-01</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>2022-06-01</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="BD1" t="inlineStr">
         <is>
           <t>2022-07-01</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="BE1" t="inlineStr">
         <is>
           <t>2022-08-01</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="BF1" t="inlineStr">
         <is>
           <t>2022-09-01</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="BG1" t="inlineStr">
         <is>
           <t>2022-10-01</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="BH1" t="inlineStr">
         <is>
           <t>2022-11-01</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="BI1" t="inlineStr">
         <is>
           <t>2022-12-01</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="BJ1" t="inlineStr">
         <is>
           <t>2023-01-01</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="BK1" t="inlineStr">
         <is>
           <t>2023-02-01</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="BL1" t="inlineStr">
         <is>
           <t>2023-03-01</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="BM1" t="inlineStr">
         <is>
           <t>2023-04-01</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="BN1" t="inlineStr">
         <is>
           <t>2023-05-01</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="BO1" t="inlineStr">
         <is>
           <t>2023-06-01</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="BP1" t="inlineStr">
         <is>
           <t>2023-07-01</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="BQ1" t="inlineStr">
         <is>
           <t>2023-08-01</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="BR1" t="inlineStr">
         <is>
           <t>2023-09-01</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="BS1" t="inlineStr">
         <is>
           <t>2023-10-01</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="BT1" t="inlineStr">
         <is>
           <t>2023-11-01</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="BU1" t="inlineStr">
         <is>
           <t>2023-12-01</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="BV1" t="inlineStr">
         <is>
           <t>2024-01-01</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="BW1" t="inlineStr">
         <is>
           <t>2024-02-01</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="BX1" t="inlineStr">
         <is>
           <t>2024-03-01</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="BY1" t="inlineStr">
         <is>
           <t>2024-04-01</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="BZ1" t="inlineStr">
         <is>
           <t>2024-05-01</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="CA1" t="inlineStr">
         <is>
           <t>2024-06-01</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="CB1" t="inlineStr">
         <is>
           <t>2024-07-01</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="CC1" t="inlineStr">
         <is>
           <t>2024-08-01</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="CD1" t="inlineStr">
         <is>
           <t>2024-09-01</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="CE1" t="inlineStr">
         <is>
           <t>2024-10-01</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="CF1" t="inlineStr">
         <is>
           <t>2024-11-01</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="CG1" t="inlineStr">
         <is>
           <t>2024-12-01</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="CH1" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="CI1" t="inlineStr">
         <is>
           <t>2025-02-01</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="CJ1" t="inlineStr">
         <is>
           <t>2025-03-01</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="CK1" t="inlineStr">
         <is>
           <t>2025-04-01</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="CL1" t="inlineStr">
         <is>
           <t>2025-05-01</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="CM1" t="inlineStr">
         <is>
           <t>2025-06-01</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="CN1" t="inlineStr">
         <is>
           <t>2025-07-01</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="CO1" t="inlineStr">
         <is>
           <t>2025-08-01</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="CP1" t="inlineStr">
         <is>
           <t>2025-09-01</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="CQ1" t="inlineStr">
         <is>
           <t>2025-10-01</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="CR1" t="inlineStr">
         <is>
           <t>2025-11-01</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="CS1" t="inlineStr">
         <is>
           <t>2025-12-01</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="CT1" t="inlineStr">
         <is>
           <t>2026-01-01</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="CU1" t="inlineStr">
         <is>
           <t>2026-02-01</t>
         </is>
       </c>
-      <c r="AZ1" t="inlineStr">
+      <c r="CV1" t="inlineStr">
         <is>
           <t>2026-03-01</t>
         </is>
       </c>
-      <c r="BA1" t="inlineStr">
+      <c r="CW1" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="BB1" t="inlineStr">
+      <c r="CX1" t="inlineStr">
         <is>
           <t>2026-05-01</t>
         </is>
       </c>
-      <c r="BC1" t="inlineStr">
+      <c r="CY1" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="BD1" t="inlineStr">
+      <c r="CZ1" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="BE1" t="inlineStr">
+      <c r="DA1" t="inlineStr">
         <is>
           <t>2026-08-01</t>
         </is>
@@ -2537,171 +2777,315 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>44168.24</v>
+      </c>
+      <c r="C2" t="n">
+        <v>44123.13</v>
+      </c>
+      <c r="D2" t="n">
+        <v>44425.37</v>
+      </c>
+      <c r="E2" t="n">
+        <v>43389.07</v>
+      </c>
+      <c r="F2" t="n">
+        <v>42591.01</v>
+      </c>
+      <c r="G2" t="n">
+        <v>42293.47</v>
+      </c>
+      <c r="H2" t="n">
+        <v>42174.45</v>
+      </c>
+      <c r="I2" t="n">
+        <v>42065.13</v>
+      </c>
+      <c r="J2" t="n">
+        <v>41745.27</v>
+      </c>
+      <c r="K2" t="n">
+        <v>41200.74</v>
+      </c>
+      <c r="L2" t="n">
+        <v>41076.6</v>
+      </c>
+      <c r="M2" t="n">
+        <v>41938.02</v>
+      </c>
+      <c r="N2" t="n">
+        <v>42063.31</v>
+      </c>
+      <c r="O2" t="n">
+        <v>41504.13</v>
+      </c>
+      <c r="P2" t="n">
+        <v>41277.22</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>41104.51</v>
+      </c>
+      <c r="R2" t="n">
+        <v>41409.45</v>
+      </c>
+      <c r="S2" t="n">
+        <v>42042.01</v>
+      </c>
+      <c r="T2" t="n">
+        <v>41370.23</v>
+      </c>
+      <c r="U2" t="n">
+        <v>41428.24</v>
+      </c>
+      <c r="V2" t="n">
+        <v>40945.95</v>
+      </c>
+      <c r="W2" t="n">
+        <v>41484.86</v>
+      </c>
+      <c r="X2" t="n">
+        <v>40965.65</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>41535.58</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>41241.73</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>41120.81</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>41241.68</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>41153.74</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>41387</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>41661.88</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>43246.88</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>43506.47</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>43052.14</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>43057.11</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>43728.23</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>44536.75</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>44072.88</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>43640.24</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>42248</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>43058.01</v>
+      </c>
+      <c r="AP2" t="n">
+        <v>43326.13</v>
+      </c>
+      <c r="AQ2" t="n">
+        <v>42385.36</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>42619.09</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>42419</v>
+      </c>
+      <c r="AT2" t="n">
+        <v>41709.65</v>
+      </c>
+      <c r="AU2" t="n">
+        <v>41276.41</v>
+      </c>
+      <c r="AV2" t="n">
+        <v>40815.97</v>
+      </c>
+      <c r="AW2" t="n">
+        <v>40736.28</v>
+      </c>
+      <c r="AX2" t="n">
         <v>40353.17</v>
       </c>
-      <c r="C2" t="n">
+      <c r="AY2" t="n">
         <v>40387.91</v>
       </c>
-      <c r="D2" t="n">
+      <c r="AZ2" t="n">
         <v>39252.17</v>
       </c>
-      <c r="E2" t="n">
+      <c r="BA2" t="n">
         <v>37053.64</v>
       </c>
-      <c r="F2" t="n">
+      <c r="BB2" t="n">
         <v>37610.21</v>
       </c>
-      <c r="G2" t="n">
+      <c r="BC2" t="n">
         <v>36273.39</v>
       </c>
-      <c r="H2" t="n">
+      <c r="BD2" t="n">
         <v>35946.73</v>
       </c>
-      <c r="I2" t="n">
+      <c r="BE2" t="n">
         <v>35098.68</v>
       </c>
-      <c r="J2" t="n">
+      <c r="BF2" t="n">
         <v>33935.23</v>
       </c>
-      <c r="K2" t="n">
+      <c r="BG2" t="n">
         <v>33821.3</v>
       </c>
-      <c r="L2" t="n">
+      <c r="BH2" t="n">
         <v>35619.67</v>
       </c>
-      <c r="M2" t="n">
+      <c r="BI2" t="n">
         <v>37208.75</v>
       </c>
-      <c r="N2" t="n">
+      <c r="BJ2" t="n">
         <v>37755.47</v>
       </c>
-      <c r="O2" t="n">
+      <c r="BK2" t="n">
         <v>36604.93</v>
       </c>
-      <c r="P2" t="n">
+      <c r="BL2" t="n">
         <v>37565.9</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="BM2" t="n">
         <v>37627.61</v>
       </c>
-      <c r="R2" t="n">
+      <c r="BN2" t="n">
         <v>36459.01</v>
       </c>
-      <c r="S2" t="n">
+      <c r="BO2" t="n">
         <v>36643.74</v>
       </c>
-      <c r="T2" t="n">
+      <c r="BP2" t="n">
         <v>37113.85</v>
       </c>
-      <c r="U2" t="n">
+      <c r="BQ2" t="n">
         <v>36448.63</v>
       </c>
-      <c r="V2" t="n">
+      <c r="BR2" t="n">
         <v>35613.44</v>
       </c>
-      <c r="W2" t="n">
+      <c r="BS2" t="n">
         <v>35213.52</v>
       </c>
-      <c r="X2" t="n">
+      <c r="BT2" t="n">
         <v>36302.63</v>
       </c>
-      <c r="Y2" t="n">
+      <c r="BU2" t="n">
         <v>37316.48</v>
       </c>
-      <c r="Z2" t="n">
+      <c r="BV2" t="n">
         <v>36438.88</v>
       </c>
-      <c r="AA2" t="n">
+      <c r="BW2" t="n">
         <v>36076.82</v>
       </c>
-      <c r="AB2" t="n">
+      <c r="BX2" t="n">
         <v>35990.22</v>
       </c>
-      <c r="AC2" t="n">
+      <c r="BY2" t="n">
         <v>35315.93</v>
       </c>
-      <c r="AD2" t="n">
+      <c r="BZ2" t="n">
         <v>35757.62</v>
       </c>
-      <c r="AE2" t="n">
+      <c r="CA2" t="n">
         <v>35242.83</v>
       </c>
-      <c r="AF2" t="n">
+      <c r="CB2" t="n">
         <v>36357.42</v>
       </c>
-      <c r="AG2" t="n">
+      <c r="CC2" t="n">
         <v>37318.04</v>
       </c>
-      <c r="AH2" t="n">
+      <c r="CD2" t="n">
         <v>37804.75</v>
       </c>
-      <c r="AI2" t="n">
+      <c r="CE2" t="n">
         <v>36337.08</v>
       </c>
-      <c r="AJ2" t="n">
+      <c r="CF2" t="n">
         <v>35805.15</v>
       </c>
-      <c r="AK2" t="n">
+      <c r="CG2" t="n">
         <v>34865.01</v>
       </c>
-      <c r="AL2" t="n">
+      <c r="CH2" t="n">
         <v>35207.95</v>
       </c>
-      <c r="AM2" t="n">
+      <c r="CI2" t="n">
         <v>35597.68</v>
       </c>
-      <c r="AN2" t="n">
+      <c r="CJ2" t="n">
         <v>36586.63</v>
       </c>
-      <c r="AO2" t="n">
+      <c r="CK2" t="n">
         <v>38564.76</v>
       </c>
-      <c r="AP2" t="n">
+      <c r="CL2" t="n">
         <v>38470.28</v>
       </c>
-      <c r="AQ2" t="n">
+      <c r="CM2" t="n">
         <v>39471.18</v>
       </c>
-      <c r="AR2" t="n">
+      <c r="CN2" t="n">
         <v>38203.05</v>
       </c>
-      <c r="AS2" t="n">
+      <c r="CO2" t="n">
         <v>39161.14</v>
       </c>
-      <c r="AT2" t="n">
+      <c r="CP2" t="n">
         <v>39204.55</v>
       </c>
-      <c r="AU2" t="n">
+      <c r="CQ2" t="n">
         <v>38314.06</v>
       </c>
-      <c r="AV2" t="n">
+      <c r="CR2" t="n">
         <v>38330</v>
       </c>
-      <c r="AW2" t="n">
+      <c r="CS2" t="n">
         <v>38641</v>
       </c>
-      <c r="AX2" t="n">
+      <c r="CT2" t="n">
         <v>39222.23</v>
       </c>
-      <c r="AY2" t="n">
+      <c r="CU2" t="n">
         <v>38992.34</v>
       </c>
-      <c r="AZ2" t="n">
+      <c r="CV2" t="n">
         <v>38121.06</v>
       </c>
-      <c r="BA2" t="n">
+      <c r="CW2" t="n">
         <v>38838</v>
       </c>
-      <c r="BB2" t="n">
+      <c r="CX2" t="n">
         <v>38587</v>
       </c>
-      <c r="BC2" t="n">
+      <c r="CY2" t="n">
         <v>37797.22</v>
       </c>
-      <c r="BD2" t="n">
+      <c r="CZ2" t="n">
         <v>38342.78</v>
       </c>
-      <c r="BE2" t="n">
+      <c r="DA2" t="n">
         <v>38577.96</v>
       </c>
     </row>
@@ -2712,152 +3096,303 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>274259.81</v>
+      </c>
+      <c r="C3" t="n">
+        <v>272844.29</v>
+      </c>
+      <c r="D3" t="n">
+        <v>284768.42</v>
+      </c>
+      <c r="E3" t="n">
+        <v>277984.08</v>
+      </c>
+      <c r="F3" t="n">
+        <v>279910.45</v>
+      </c>
+      <c r="G3" t="n">
+        <v>284337.09</v>
+      </c>
+      <c r="H3" t="n">
+        <v>278827.29</v>
+      </c>
+      <c r="I3" t="n">
+        <v>282274.78</v>
+      </c>
+      <c r="J3" t="n">
+        <v>283668.66</v>
+      </c>
+      <c r="K3" t="n">
+        <v>280712.83</v>
+      </c>
+      <c r="L3" t="n">
+        <v>284725.34</v>
+      </c>
+      <c r="M3" t="n">
+        <v>289855.95</v>
+      </c>
+      <c r="N3" t="n">
+        <v>289000.01</v>
+      </c>
+      <c r="O3" t="n">
+        <v>287731.42</v>
+      </c>
+      <c r="P3" t="n">
+        <v>291618.3</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>294223.54</v>
+      </c>
+      <c r="R3" t="n">
+        <v>297243.68</v>
+      </c>
+      <c r="S3" t="n">
+        <v>296488.58</v>
+      </c>
+      <c r="T3" t="n">
+        <v>301577.12</v>
+      </c>
+      <c r="U3" t="n">
+        <v>303114.73</v>
+      </c>
+      <c r="V3" t="n">
+        <v>296303.53</v>
+      </c>
+      <c r="W3" t="n">
+        <v>297636.32</v>
+      </c>
+      <c r="X3" t="n">
+        <v>293922.92</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>296226.05</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>295315</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>296666</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>303885</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>304849</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>306422</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>306298</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>309633</v>
+      </c>
+      <c r="AG3" t="n">
+        <v>312504</v>
+      </c>
+      <c r="AH3" t="n">
+        <v>312897</v>
+      </c>
+      <c r="AI3" t="n">
+        <v>316925</v>
+      </c>
+      <c r="AJ3" t="n">
+        <v>315802</v>
+      </c>
+      <c r="AK3" t="n">
+        <v>317741</v>
+      </c>
+      <c r="AL3" t="n">
+        <v>315565</v>
+      </c>
+      <c r="AM3" t="n">
+        <v>313529</v>
+      </c>
+      <c r="AN3" t="n">
+        <v>310995</v>
+      </c>
+      <c r="AO3" t="n">
+        <v>314363</v>
+      </c>
+      <c r="AP3" t="n">
+        <v>317055</v>
+      </c>
+      <c r="AQ3" t="n">
+        <v>319843</v>
+      </c>
+      <c r="AR3" t="n">
+        <v>319949</v>
+      </c>
+      <c r="AS3" t="n">
+        <v>319061</v>
+      </c>
+      <c r="AT3" t="n">
+        <v>316468</v>
+      </c>
+      <c r="AU3" t="n">
+        <v>318692</v>
+      </c>
+      <c r="AV3" t="n">
+        <v>319708</v>
+      </c>
+      <c r="AW3" t="n">
+        <v>318170</v>
+      </c>
+      <c r="AX3" t="n">
         <v>312546</v>
       </c>
-      <c r="C3" t="n">
+      <c r="AY3" t="n">
         <v>313471</v>
       </c>
-      <c r="D3" t="n">
+      <c r="AZ3" t="n">
         <v>309506</v>
       </c>
-      <c r="E3" t="n">
+      <c r="BA3" t="n">
         <v>305206</v>
       </c>
-      <c r="F3" t="n">
+      <c r="BB3" t="n">
         <v>307840</v>
       </c>
-      <c r="G3" t="n">
+      <c r="BC3" t="n">
         <v>305918</v>
       </c>
-      <c r="H3" t="n">
+      <c r="BD3" t="n">
         <v>308938</v>
       </c>
-      <c r="I3" t="n">
+      <c r="BE3" t="n">
         <v>306005</v>
       </c>
-      <c r="J3" t="n">
+      <c r="BF3" t="n">
         <v>303179</v>
       </c>
-      <c r="K3" t="n">
+      <c r="BG3" t="n">
         <v>304221</v>
       </c>
-      <c r="L3" t="n">
+      <c r="BH3" t="n">
         <v>309061</v>
       </c>
-      <c r="M3" t="n">
+      <c r="BI3" t="n">
         <v>315345</v>
       </c>
-      <c r="N3" t="n">
+      <c r="BJ3" t="n">
         <v>310949</v>
       </c>
-      <c r="O3" t="n">
+      <c r="BK3" t="n">
         <v>293900</v>
       </c>
-      <c r="P3" t="n">
+      <c r="BL3" t="n">
         <v>297950</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="BM3" t="n">
         <v>295116</v>
       </c>
-      <c r="R3" t="n">
+      <c r="BN3" t="n">
         <v>292792</v>
       </c>
-      <c r="S3" t="n">
+      <c r="BO3" t="n">
         <v>293016</v>
       </c>
-      <c r="T3" t="n">
+      <c r="BP3" t="n">
         <v>294678</v>
       </c>
-      <c r="U3" t="n">
+      <c r="BQ3" t="n">
         <v>292405</v>
       </c>
-      <c r="V3" t="n">
+      <c r="BR3" t="n">
         <v>285245</v>
       </c>
-      <c r="W3" t="n">
+      <c r="BS3" t="n">
         <v>287457</v>
       </c>
-      <c r="X3" t="n">
+      <c r="BT3" t="n">
         <v>295267</v>
       </c>
-      <c r="Y3" t="n">
+      <c r="BU3" t="n">
         <v>301470</v>
       </c>
-      <c r="Z3" t="n">
+      <c r="BV3" t="n">
         <v>299104</v>
       </c>
-      <c r="AA3" t="n">
+      <c r="BW3" t="n">
         <v>298787</v>
       </c>
-      <c r="AB3" t="n">
+      <c r="BX3" t="n">
         <v>298344</v>
       </c>
-      <c r="AC3" t="n">
+      <c r="BY3" t="n">
         <v>295492</v>
       </c>
-      <c r="AD3" t="n">
+      <c r="BZ3" t="n">
         <v>298861</v>
       </c>
-      <c r="AE3" t="n">
+      <c r="CA3" t="n">
         <v>301235</v>
       </c>
-      <c r="AF3" t="n">
+      <c r="CB3" t="n">
         <v>301245</v>
       </c>
-      <c r="AG3" t="n">
+      <c r="CC3" t="n">
         <v>300873</v>
       </c>
-      <c r="AH3" t="n">
+      <c r="CD3" t="n">
         <v>303818</v>
       </c>
-      <c r="AI3" t="n">
+      <c r="CE3" t="n">
         <v>299382</v>
       </c>
-      <c r="AJ3" t="n">
+      <c r="CF3" t="n">
         <v>300478</v>
       </c>
-      <c r="AK3" t="n">
+      <c r="CG3" t="n">
         <v>300657</v>
       </c>
-      <c r="AL3" t="n">
+      <c r="CH3" t="n">
         <v>298104</v>
       </c>
-      <c r="AM3" t="n">
+      <c r="CI3" t="n">
         <v>302136</v>
       </c>
-      <c r="AN3" t="n">
+      <c r="CJ3" t="n">
         <v>304980</v>
       </c>
-      <c r="AO3" t="n">
+      <c r="CK3" t="n">
         <v>310594</v>
       </c>
-      <c r="AP3" t="n">
+      <c r="CL3" t="n">
         <v>312792</v>
       </c>
-      <c r="AQ3" t="n">
+      <c r="CM3" t="n">
         <v>316343</v>
       </c>
-      <c r="AR3" t="n">
+      <c r="CN3" t="n">
         <v>314415</v>
       </c>
-      <c r="AS3" t="n">
+      <c r="CO3" t="n">
         <v>316890</v>
       </c>
-      <c r="AT3" t="n">
+      <c r="CP3" t="n">
         <v>322760</v>
       </c>
-      <c r="AU3" t="n">
+      <c r="CQ3" t="n">
         <v>322351</v>
       </c>
-      <c r="AV3" t="n">
+      <c r="CR3" t="n">
         <v>325548</v>
       </c>
-      <c r="AW3" t="n">
+      <c r="CS3" t="n">
         <v>334436</v>
       </c>
-      <c r="AX3" t="n">
+      <c r="CT3" t="n">
         <v>336577</v>
       </c>
+      <c r="CU3" t="inlineStr"/>
+      <c r="CV3" t="inlineStr"/>
+      <c r="CW3" t="inlineStr"/>
+      <c r="CX3" t="inlineStr"/>
+      <c r="CY3" t="inlineStr"/>
+      <c r="CZ3" t="inlineStr"/>
+      <c r="DA3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2866,171 +3401,315 @@
         </is>
       </c>
       <c r="B4" t="n">
+        <v>1205293</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1199398</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1205697</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1194057</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1193135</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1198018</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1196341</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1199809</v>
+      </c>
+      <c r="J4" t="n">
+        <v>1200678</v>
+      </c>
+      <c r="K4" t="n">
+        <v>1193097</v>
+      </c>
+      <c r="L4" t="n">
+        <v>1198375</v>
+      </c>
+      <c r="M4" t="n">
+        <v>1209496</v>
+      </c>
+      <c r="N4" t="n">
+        <v>1216661</v>
+      </c>
+      <c r="O4" t="n">
+        <v>1219313</v>
+      </c>
+      <c r="P4" t="n">
+        <v>1229960</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>1230402</v>
+      </c>
+      <c r="R4" t="n">
+        <v>1244731</v>
+      </c>
+      <c r="S4" t="n">
+        <v>1256444</v>
+      </c>
+      <c r="T4" t="n">
+        <v>1250592</v>
+      </c>
+      <c r="U4" t="n">
+        <v>1263371</v>
+      </c>
+      <c r="V4" t="n">
+        <v>1255607</v>
+      </c>
+      <c r="W4" t="n">
+        <v>1256451</v>
+      </c>
+      <c r="X4" t="n">
+        <v>1251522</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>1255903</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>1273044</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>1289285</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>1296725</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>1295381</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>1303715</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>1306500</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>1319927</v>
+      </c>
+      <c r="AG4" t="n">
+        <v>1316046</v>
+      </c>
+      <c r="AH4" t="n">
+        <v>1309429</v>
+      </c>
+      <c r="AI4" t="n">
+        <v>1304050</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>1306781</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>1312792</v>
+      </c>
+      <c r="AL4" t="n">
+        <v>1310835</v>
+      </c>
+      <c r="AM4" t="n">
+        <v>1301199</v>
+      </c>
+      <c r="AN4" t="n">
+        <v>1288353</v>
+      </c>
+      <c r="AO4" t="n">
+        <v>1295819</v>
+      </c>
+      <c r="AP4" t="n">
+        <v>1301051</v>
+      </c>
+      <c r="AQ4" t="n">
+        <v>1294260</v>
+      </c>
+      <c r="AR4" t="n">
+        <v>1302526</v>
+      </c>
+      <c r="AS4" t="n">
+        <v>1298637</v>
+      </c>
+      <c r="AT4" t="n">
+        <v>1285508</v>
+      </c>
+      <c r="AU4" t="n">
+        <v>1279041</v>
+      </c>
+      <c r="AV4" t="n">
+        <v>1283852</v>
+      </c>
+      <c r="AW4" t="n">
+        <v>1283272</v>
+      </c>
+      <c r="AX4" t="n">
         <v>1264244</v>
       </c>
-      <c r="C4" t="n">
+      <c r="AY4" t="n">
         <v>1259159</v>
       </c>
-      <c r="D4" t="n">
+      <c r="AZ4" t="n">
         <v>1230520</v>
       </c>
-      <c r="E4" t="n">
+      <c r="BA4" t="n">
         <v>1199561</v>
       </c>
-      <c r="F4" t="n">
+      <c r="BB4" t="n">
         <v>1208699</v>
       </c>
-      <c r="G4" t="n">
+      <c r="BC4" t="n">
         <v>1192911</v>
       </c>
-      <c r="H4" t="n">
+      <c r="BD4" t="n">
         <v>1206630</v>
       </c>
-      <c r="I4" t="n">
+      <c r="BE4" t="n">
         <v>1176896</v>
       </c>
-      <c r="J4" t="n">
+      <c r="BF4" t="n">
         <v>1125304</v>
       </c>
-      <c r="K4" t="n">
+      <c r="BG4" t="n">
         <v>1082452</v>
       </c>
-      <c r="L4" t="n">
+      <c r="BH4" t="n">
         <v>1109364</v>
       </c>
-      <c r="M4" t="n">
+      <c r="BI4" t="n">
         <v>1108189</v>
       </c>
-      <c r="N4" t="n">
+      <c r="BJ4" t="n">
         <v>1126868</v>
       </c>
-      <c r="O4" t="n">
+      <c r="BK4" t="n">
         <v>1106343</v>
       </c>
-      <c r="P4" t="n">
+      <c r="BL4" t="n">
         <v>1134005</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="BM4" t="n">
         <v>1142230</v>
       </c>
-      <c r="R4" t="n">
+      <c r="BN4" t="n">
         <v>1132162</v>
       </c>
-      <c r="S4" t="n">
+      <c r="BO4" t="n">
         <v>1126104</v>
       </c>
-      <c r="T4" t="n">
+      <c r="BP4" t="n">
         <v>1130301</v>
       </c>
-      <c r="U4" t="n">
+      <c r="BQ4" t="n">
         <v>1132621</v>
       </c>
-      <c r="V4" t="n">
+      <c r="BR4" t="n">
         <v>1120048</v>
       </c>
-      <c r="W4" t="n">
+      <c r="BS4" t="n">
         <v>1117193</v>
       </c>
-      <c r="X4" t="n">
+      <c r="BT4" t="n">
         <v>1146719</v>
       </c>
-      <c r="Y4" t="n">
+      <c r="BU4" t="n">
         <v>1170437</v>
       </c>
-      <c r="Z4" t="n">
+      <c r="BV4" t="n">
         <v>1169506</v>
       </c>
-      <c r="AA4" t="n">
+      <c r="BW4" t="n">
         <v>1158491</v>
       </c>
-      <c r="AB4" t="n">
+      <c r="BX4" t="n">
         <v>1163521</v>
       </c>
-      <c r="AC4" t="n">
+      <c r="BY4" t="n">
         <v>1149316</v>
       </c>
-      <c r="AD4" t="n">
+      <c r="BZ4" t="n">
         <v>1100113</v>
       </c>
-      <c r="AE4" t="n">
+      <c r="CA4" t="n">
         <v>1100691</v>
       </c>
-      <c r="AF4" t="n">
+      <c r="CB4" t="n">
         <v>1084573</v>
       </c>
-      <c r="AG4" t="n">
+      <c r="CC4" t="n">
         <v>1097528</v>
       </c>
-      <c r="AH4" t="n">
+      <c r="CD4" t="n">
         <v>1112931</v>
       </c>
-      <c r="AI4" t="n">
+      <c r="CE4" t="n">
         <v>1095601</v>
       </c>
-      <c r="AJ4" t="n">
+      <c r="CF4" t="n">
         <v>1099052</v>
       </c>
-      <c r="AK4" t="n">
+      <c r="CG4" t="n">
         <v>1092306</v>
       </c>
-      <c r="AL4" t="n">
+      <c r="CH4" t="n">
         <v>1096788</v>
       </c>
-      <c r="AM4" t="n">
+      <c r="CI4" t="n">
         <v>1108410</v>
       </c>
-      <c r="AN4" t="n">
+      <c r="CJ4" t="n">
         <v>1118981</v>
       </c>
-      <c r="AO4" t="n">
+      <c r="CK4" t="n">
         <v>1136746</v>
       </c>
-      <c r="AP4" t="n">
+      <c r="CL4" t="n">
         <v>1137098</v>
       </c>
-      <c r="AQ4" t="n">
+      <c r="CM4" t="n">
         <v>1151692</v>
       </c>
-      <c r="AR4" t="n">
+      <c r="CN4" t="n">
         <v>1143537</v>
       </c>
-      <c r="AS4" t="n">
+      <c r="CO4" t="n">
         <v>1158765</v>
       </c>
-      <c r="AT4" t="n">
+      <c r="CP4" t="n">
         <v>1165059</v>
       </c>
-      <c r="AU4" t="n">
+      <c r="CQ4" t="n">
         <v>1166724</v>
       </c>
-      <c r="AV4" t="n">
+      <c r="CR4" t="n">
         <v>1173675</v>
       </c>
-      <c r="AW4" t="n">
+      <c r="CS4" t="n">
         <v>1180501</v>
       </c>
-      <c r="AX4" t="n">
+      <c r="CT4" t="n">
         <v>1186456</v>
       </c>
-      <c r="AY4" t="n">
+      <c r="CU4" t="n">
         <v>1196112</v>
       </c>
-      <c r="AZ4" t="n">
+      <c r="CV4" t="n">
         <v>1177807</v>
       </c>
-      <c r="BA4" t="n">
+      <c r="CW4" t="n">
         <v>1185255</v>
       </c>
-      <c r="BB4" t="n">
+      <c r="CX4" t="n">
         <v>1109822</v>
       </c>
-      <c r="BC4" t="n">
+      <c r="CY4" t="n">
         <v>1106270</v>
       </c>
-      <c r="BD4" t="n">
+      <c r="CZ4" t="n">
         <v>1105474</v>
       </c>
-      <c r="BE4" t="n">
+      <c r="DA4" t="n">
         <v>1010831</v>
       </c>
     </row>
@@ -3041,171 +3720,315 @@
         </is>
       </c>
       <c r="B5" t="n">
+        <v>125461.87</v>
+      </c>
+      <c r="C5" t="n">
+        <v>123521.13</v>
+      </c>
+      <c r="D5" t="n">
+        <v>126576.95</v>
+      </c>
+      <c r="E5" t="n">
+        <v>124055.98</v>
+      </c>
+      <c r="F5" t="n">
+        <v>128025.18</v>
+      </c>
+      <c r="G5" t="n">
+        <v>124617.12</v>
+      </c>
+      <c r="H5" t="n">
+        <v>121881.65</v>
+      </c>
+      <c r="I5" t="n">
+        <v>127225.85</v>
+      </c>
+      <c r="J5" t="n">
+        <v>122815.8</v>
+      </c>
+      <c r="K5" t="n">
+        <v>125831.34</v>
+      </c>
+      <c r="L5" t="n">
+        <v>135365.54</v>
+      </c>
+      <c r="M5" t="n">
+        <v>140168.14</v>
+      </c>
+      <c r="N5" t="n">
+        <v>141779.55</v>
+      </c>
+      <c r="O5" t="n">
+        <v>136435.91</v>
+      </c>
+      <c r="P5" t="n">
+        <v>130417.48</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>133217.12</v>
+      </c>
+      <c r="R5" t="n">
+        <v>122583.15</v>
+      </c>
+      <c r="S5" t="n">
+        <v>125604.33</v>
+      </c>
+      <c r="T5" t="n">
+        <v>132772</v>
+      </c>
+      <c r="U5" t="n">
+        <v>131317.36</v>
+      </c>
+      <c r="V5" t="n">
+        <v>123048.55</v>
+      </c>
+      <c r="W5" t="n">
+        <v>138785.16</v>
+      </c>
+      <c r="X5" t="n">
+        <v>134468.6</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>137539.03</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>132885.96</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>130309.07</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>133655.07</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>135854.68</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>136562.64</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>134910.99</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>136989.92</v>
+      </c>
+      <c r="AG5" t="n">
+        <v>135827</v>
+      </c>
+      <c r="AH5" t="n">
+        <v>129374.75</v>
+      </c>
+      <c r="AI5" t="n">
+        <v>132254.18</v>
+      </c>
+      <c r="AJ5" t="n">
+        <v>139974.47</v>
+      </c>
+      <c r="AK5" t="n">
+        <v>139604.9</v>
+      </c>
+      <c r="AL5" t="n">
+        <v>133428.36</v>
+      </c>
+      <c r="AM5" t="n">
+        <v>132396.65</v>
+      </c>
+      <c r="AN5" t="n">
+        <v>133257.24</v>
+      </c>
+      <c r="AO5" t="n">
+        <v>133111.17</v>
+      </c>
+      <c r="AP5" t="n">
+        <v>130867.43</v>
+      </c>
+      <c r="AQ5" t="n">
+        <v>129543.66</v>
+      </c>
+      <c r="AR5" t="n">
+        <v>130947.23</v>
+      </c>
+      <c r="AS5" t="n">
+        <v>126172.45</v>
+      </c>
+      <c r="AT5" t="n">
+        <v>127854.28</v>
+      </c>
+      <c r="AU5" t="n">
+        <v>126013.69</v>
+      </c>
+      <c r="AV5" t="n">
+        <v>126818.82</v>
+      </c>
+      <c r="AW5" t="n">
+        <v>127803.59</v>
+      </c>
+      <c r="AX5" t="n">
         <v>120411.92</v>
       </c>
-      <c r="C5" t="n">
+      <c r="AY5" t="n">
         <v>120532.75</v>
       </c>
-      <c r="D5" t="n">
+      <c r="AZ5" t="n">
         <v>123104.96</v>
       </c>
-      <c r="E5" t="n">
+      <c r="BA5" t="n">
         <v>115053.03</v>
       </c>
-      <c r="F5" t="n">
+      <c r="BB5" t="n">
         <v>112608.82</v>
       </c>
-      <c r="G5" t="n">
+      <c r="BC5" t="n">
         <v>110336.99</v>
       </c>
-      <c r="H5" t="n">
+      <c r="BD5" t="n">
         <v>108203.65</v>
       </c>
-      <c r="I5" t="n">
+      <c r="BE5" t="n">
         <v>107780.62</v>
       </c>
-      <c r="J5" t="n">
+      <c r="BF5" t="n">
         <v>97646.82000000001</v>
       </c>
-      <c r="K5" t="n">
+      <c r="BG5" t="n">
         <v>101927.45</v>
       </c>
-      <c r="L5" t="n">
+      <c r="BH5" t="n">
         <v>108268.35</v>
       </c>
-      <c r="M5" t="n">
+      <c r="BI5" t="n">
         <v>110285.51</v>
       </c>
-      <c r="N5" t="n">
+      <c r="BJ5" t="n">
         <v>108424.78</v>
       </c>
-      <c r="O5" t="n">
+      <c r="BK5" t="n">
         <v>102781.8</v>
       </c>
-      <c r="P5" t="n">
+      <c r="BL5" t="n">
         <v>105046.47</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="BM5" t="n">
         <v>107719.01</v>
       </c>
-      <c r="R5" t="n">
+      <c r="BN5" t="n">
         <v>104068.46</v>
       </c>
-      <c r="S5" t="n">
+      <c r="BO5" t="n">
         <v>106042.77</v>
       </c>
-      <c r="T5" t="n">
+      <c r="BP5" t="n">
         <v>110108.85</v>
       </c>
-      <c r="U5" t="n">
+      <c r="BQ5" t="n">
         <v>109175.59</v>
       </c>
-      <c r="V5" t="n">
+      <c r="BR5" t="n">
         <v>103971.13</v>
       </c>
-      <c r="W5" t="n">
+      <c r="BS5" t="n">
         <v>103736.91</v>
       </c>
-      <c r="X5" t="n">
+      <c r="BT5" t="n">
         <v>106107.64</v>
       </c>
-      <c r="Y5" t="n">
+      <c r="BU5" t="n">
         <v>108765.24</v>
       </c>
-      <c r="Z5" t="n">
+      <c r="BV5" t="n">
         <v>105698.52</v>
       </c>
-      <c r="AA5" t="n">
+      <c r="BW5" t="n">
         <v>104694.58</v>
       </c>
-      <c r="AB5" t="n">
+      <c r="BX5" t="n">
         <v>105493.85</v>
       </c>
-      <c r="AC5" t="n">
+      <c r="BY5" t="n">
         <v>100104.93</v>
       </c>
-      <c r="AD5" t="n">
+      <c r="BZ5" t="n">
         <v>103539.63</v>
       </c>
-      <c r="AE5" t="n">
+      <c r="CA5" t="n">
         <v>102150.43</v>
       </c>
-      <c r="AF5" t="n">
+      <c r="CB5" t="n">
         <v>106238.07</v>
       </c>
-      <c r="AG5" t="n">
+      <c r="CC5" t="n">
         <v>107970.45</v>
       </c>
-      <c r="AH5" t="n">
+      <c r="CD5" t="n">
         <v>106798.85</v>
       </c>
-      <c r="AI5" t="n">
+      <c r="CE5" t="n">
         <v>104268.48</v>
       </c>
-      <c r="AJ5" t="n">
+      <c r="CF5" t="n">
         <v>104730.56</v>
       </c>
-      <c r="AK5" t="n">
+      <c r="CG5" t="n">
         <v>102683.2</v>
       </c>
-      <c r="AL5" t="n">
+      <c r="CH5" t="n">
         <v>102719.52</v>
       </c>
-      <c r="AM5" t="n">
+      <c r="CI5" t="n">
         <v>104175.92</v>
       </c>
-      <c r="AN5" t="n">
+      <c r="CJ5" t="n">
         <v>106345.15</v>
       </c>
-      <c r="AO5" t="n">
+      <c r="CK5" t="n">
         <v>111229.13</v>
       </c>
-      <c r="AP5" t="n">
+      <c r="CL5" t="n">
         <v>112666.82</v>
       </c>
-      <c r="AQ5" t="n">
+      <c r="CM5" t="n">
         <v>116903.29</v>
       </c>
-      <c r="AR5" t="n">
+      <c r="CN5" t="n">
         <v>115962.86</v>
       </c>
-      <c r="AS5" t="n">
+      <c r="CO5" t="n">
         <v>118608.23</v>
       </c>
-      <c r="AT5" t="n">
+      <c r="CP5" t="n">
         <v>122086.56</v>
       </c>
-      <c r="AU5" t="n">
+      <c r="CQ5" t="n">
         <v>121043.62</v>
       </c>
-      <c r="AV5" t="n">
+      <c r="CR5" t="n">
         <v>123015.11</v>
       </c>
-      <c r="AW5" t="n">
+      <c r="CS5" t="n">
         <v>123790.23</v>
       </c>
-      <c r="AX5" t="n">
+      <c r="CT5" t="n">
         <v>123927.95</v>
       </c>
-      <c r="AY5" t="n">
+      <c r="CU5" t="n">
         <v>126625.3</v>
       </c>
-      <c r="AZ5" t="n">
+      <c r="CV5" t="n">
         <v>126449.82</v>
       </c>
-      <c r="BA5" t="n">
+      <c r="CW5" t="n">
         <v>122681.06</v>
       </c>
-      <c r="BB5" t="n">
+      <c r="CX5" t="n">
         <v>123400.43</v>
       </c>
-      <c r="BC5" t="n">
+      <c r="CY5" t="n">
         <v>129270.91</v>
       </c>
-      <c r="BD5" t="n">
+      <c r="CZ5" t="n">
         <v>122614.11</v>
       </c>
-      <c r="BE5" t="n">
+      <c r="DA5" t="n">
         <v>123120.95</v>
       </c>
     </row>
@@ -3216,171 +4039,315 @@
         </is>
       </c>
       <c r="B6" t="n">
+        <v>44405</v>
+      </c>
+      <c r="C6" t="n">
+        <v>47225</v>
+      </c>
+      <c r="D6" t="n">
+        <v>50587</v>
+      </c>
+      <c r="E6" t="n">
+        <v>46524</v>
+      </c>
+      <c r="F6" t="n">
+        <v>54243</v>
+      </c>
+      <c r="G6" t="n">
+        <v>47575</v>
+      </c>
+      <c r="H6" t="n">
+        <v>42577</v>
+      </c>
+      <c r="I6" t="n">
+        <v>42964</v>
+      </c>
+      <c r="J6" t="n">
+        <v>44401</v>
+      </c>
+      <c r="K6" t="n">
+        <v>36672</v>
+      </c>
+      <c r="L6" t="n">
+        <v>39589</v>
+      </c>
+      <c r="M6" t="n">
+        <v>45406</v>
+      </c>
+      <c r="N6" t="n">
+        <v>35709</v>
+      </c>
+      <c r="O6" t="n">
+        <v>39748</v>
+      </c>
+      <c r="P6" t="n">
+        <v>45576</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>44222</v>
+      </c>
+      <c r="R6" t="n">
+        <v>46181</v>
+      </c>
+      <c r="S6" t="n">
+        <v>45253</v>
+      </c>
+      <c r="T6" t="n">
+        <v>35518</v>
+      </c>
+      <c r="U6" t="n">
+        <v>38978</v>
+      </c>
+      <c r="V6" t="n">
+        <v>36838</v>
+      </c>
+      <c r="W6" t="n">
+        <v>38062</v>
+      </c>
+      <c r="X6" t="n">
+        <v>42742</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>49688</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>39830</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>44930</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>46901</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>31571</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>30195</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>32012</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>32915</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>33035</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>32450</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>32341</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>32949</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>32128</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>31088</v>
+      </c>
+      <c r="AM6" t="n">
+        <v>32952</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>36814</v>
+      </c>
+      <c r="AO6" t="n">
+        <v>36229</v>
+      </c>
+      <c r="AP6" t="n">
+        <v>35704</v>
+      </c>
+      <c r="AQ6" t="n">
+        <v>37302</v>
+      </c>
+      <c r="AR6" t="n">
+        <v>35766</v>
+      </c>
+      <c r="AS6" t="n">
+        <v>37427</v>
+      </c>
+      <c r="AT6" t="n">
+        <v>38206</v>
+      </c>
+      <c r="AU6" t="n">
+        <v>35968</v>
+      </c>
+      <c r="AV6" t="n">
+        <v>37011</v>
+      </c>
+      <c r="AW6" t="n">
+        <v>37425</v>
+      </c>
+      <c r="AX6" t="n">
         <v>35902</v>
       </c>
-      <c r="C6" t="n">
+      <c r="AY6" t="n">
         <v>36120</v>
       </c>
-      <c r="D6" t="n">
+      <c r="AZ6" t="n">
         <v>36276</v>
       </c>
-      <c r="E6" t="n">
+      <c r="BA6" t="n">
         <v>34607</v>
       </c>
-      <c r="F6" t="n">
+      <c r="BB6" t="n">
         <v>35095</v>
       </c>
-      <c r="G6" t="n">
+      <c r="BC6" t="n">
         <v>34447</v>
       </c>
-      <c r="H6" t="n">
+      <c r="BD6" t="n">
         <v>35634</v>
       </c>
-      <c r="I6" t="n">
+      <c r="BE6" t="n">
         <v>35922</v>
       </c>
-      <c r="J6" t="n">
+      <c r="BF6" t="n">
         <v>35037</v>
       </c>
-      <c r="K6" t="n">
+      <c r="BG6" t="n">
         <v>36113</v>
       </c>
-      <c r="L6" t="n">
+      <c r="BH6" t="n">
         <v>39040</v>
       </c>
-      <c r="M6" t="n">
+      <c r="BI6" t="n">
         <v>38480</v>
       </c>
-      <c r="N6" t="n">
+      <c r="BJ6" t="n">
         <v>38149</v>
       </c>
-      <c r="O6" t="n">
+      <c r="BK6" t="n">
         <v>35320</v>
       </c>
-      <c r="P6" t="n">
+      <c r="BL6" t="n">
         <v>36375</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="BM6" t="n">
         <v>38679</v>
       </c>
-      <c r="R6" t="n">
+      <c r="BN6" t="n">
         <v>36115</v>
       </c>
-      <c r="S6" t="n">
+      <c r="BO6" t="n">
         <v>36911</v>
       </c>
-      <c r="T6" t="n">
+      <c r="BP6" t="n">
         <v>38215</v>
       </c>
-      <c r="U6" t="n">
+      <c r="BQ6" t="n">
         <v>38434</v>
       </c>
-      <c r="V6" t="n">
+      <c r="BR6" t="n">
         <v>35744</v>
       </c>
-      <c r="W6" t="n">
+      <c r="BS6" t="n">
         <v>35888</v>
       </c>
-      <c r="X6" t="n">
+      <c r="BT6" t="n">
         <v>38009</v>
       </c>
-      <c r="Y6" t="n">
+      <c r="BU6" t="n">
         <v>40897</v>
       </c>
-      <c r="Z6" t="n">
+      <c r="BV6" t="n">
         <v>35026</v>
       </c>
-      <c r="AA6" t="n">
+      <c r="BW6" t="n">
         <v>35126</v>
       </c>
-      <c r="AB6" t="n">
+      <c r="BX6" t="n">
         <v>34212</v>
       </c>
-      <c r="AC6" t="n">
+      <c r="BY6" t="n">
         <v>33803</v>
       </c>
-      <c r="AD6" t="n">
+      <c r="BZ6" t="n">
         <v>35618</v>
       </c>
-      <c r="AE6" t="n">
+      <c r="CA6" t="n">
         <v>37644</v>
       </c>
-      <c r="AF6" t="n">
+      <c r="CB6" t="n">
         <v>36729</v>
       </c>
-      <c r="AG6" t="n">
+      <c r="CC6" t="n">
         <v>40610</v>
       </c>
-      <c r="AH6" t="n">
+      <c r="CD6" t="n">
         <v>39957</v>
       </c>
-      <c r="AI6" t="n">
+      <c r="CE6" t="n">
         <v>39030</v>
       </c>
-      <c r="AJ6" t="n">
+      <c r="CF6" t="n">
         <v>39287</v>
       </c>
-      <c r="AK6" t="n">
+      <c r="CG6" t="n">
         <v>39576</v>
       </c>
-      <c r="AL6" t="n">
+      <c r="CH6" t="n">
         <v>40770</v>
       </c>
-      <c r="AM6" t="n">
+      <c r="CI6" t="n">
         <v>41970</v>
       </c>
-      <c r="AN6" t="n">
+      <c r="CJ6" t="n">
         <v>41098</v>
       </c>
-      <c r="AO6" t="n">
+      <c r="CK6" t="n">
         <v>39891</v>
       </c>
-      <c r="AP6" t="n">
+      <c r="CL6" t="n">
         <v>41757</v>
       </c>
-      <c r="AQ6" t="n">
+      <c r="CM6" t="n">
         <v>39970</v>
       </c>
-      <c r="AR6" t="n">
+      <c r="CN6" t="n">
         <v>39476</v>
       </c>
-      <c r="AS6" t="n">
+      <c r="CO6" t="n">
         <v>40717</v>
       </c>
-      <c r="AT6" t="n">
+      <c r="CP6" t="n">
         <v>42175</v>
       </c>
-      <c r="AU6" t="n">
+      <c r="CQ6" t="n">
         <v>41482</v>
       </c>
-      <c r="AV6" t="n">
+      <c r="CR6" t="n">
         <v>42782</v>
       </c>
-      <c r="AW6" t="n">
+      <c r="CS6" t="n">
         <v>44962</v>
       </c>
-      <c r="AX6" t="n">
+      <c r="CT6" t="n">
         <v>40964</v>
       </c>
-      <c r="AY6" t="n">
+      <c r="CU6" t="n">
         <v>42106</v>
       </c>
-      <c r="AZ6" t="n">
+      <c r="CV6" t="n">
         <v>41982</v>
       </c>
-      <c r="BA6" t="n">
+      <c r="CW6" t="n">
         <v>41544</v>
       </c>
-      <c r="BB6" t="n">
+      <c r="CX6" t="n">
         <v>40705</v>
       </c>
-      <c r="BC6" t="n">
+      <c r="CY6" t="n">
         <v>40914</v>
       </c>
-      <c r="BD6" t="n">
+      <c r="CZ6" t="n">
         <v>46176</v>
       </c>
-      <c r="BE6" t="n">
+      <c r="DA6" t="n">
         <v>45499</v>
       </c>
     </row>
@@ -3391,171 +4358,315 @@
         </is>
       </c>
       <c r="B7" t="n">
+        <v>76504</v>
+      </c>
+      <c r="C7" t="n">
+        <v>76284</v>
+      </c>
+      <c r="D7" t="n">
+        <v>73045</v>
+      </c>
+      <c r="E7" t="n">
+        <v>72085</v>
+      </c>
+      <c r="F7" t="n">
+        <v>70791</v>
+      </c>
+      <c r="G7" t="n">
+        <v>71453</v>
+      </c>
+      <c r="H7" t="n">
+        <v>71500</v>
+      </c>
+      <c r="I7" t="n">
+        <v>70944</v>
+      </c>
+      <c r="J7" t="n">
+        <v>70434</v>
+      </c>
+      <c r="K7" t="n">
+        <v>71742</v>
+      </c>
+      <c r="L7" t="n">
+        <v>71635</v>
+      </c>
+      <c r="M7" t="n">
+        <v>73279</v>
+      </c>
+      <c r="N7" t="n">
+        <v>76908</v>
+      </c>
+      <c r="O7" t="n">
+        <v>73482</v>
+      </c>
+      <c r="P7" t="n">
+        <v>72539</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>74610</v>
+      </c>
+      <c r="R7" t="n">
+        <v>74403</v>
+      </c>
+      <c r="S7" t="n">
+        <v>74927</v>
+      </c>
+      <c r="T7" t="n">
+        <v>73768</v>
+      </c>
+      <c r="U7" t="n">
+        <v>74708</v>
+      </c>
+      <c r="V7" t="n">
+        <v>73841</v>
+      </c>
+      <c r="W7" t="n">
+        <v>73983</v>
+      </c>
+      <c r="X7" t="n">
+        <v>73421</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>73613</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>74837</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>75995</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>74610</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>75551</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>75215</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>74696</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>77469</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>76909</v>
+      </c>
+      <c r="AH7" t="n">
+        <v>77316</v>
+      </c>
+      <c r="AI7" t="n">
+        <v>77782</v>
+      </c>
+      <c r="AJ7" t="n">
+        <v>78480</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>76820</v>
+      </c>
+      <c r="AL7" t="n">
+        <v>75673</v>
+      </c>
+      <c r="AM7" t="n">
+        <v>72917</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>70253</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>71109</v>
+      </c>
+      <c r="AP7" t="n">
+        <v>76049</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>75938</v>
+      </c>
+      <c r="AR7" t="n">
+        <v>77013</v>
+      </c>
+      <c r="AS7" t="n">
+        <v>77961</v>
+      </c>
+      <c r="AT7" t="n">
+        <v>77935</v>
+      </c>
+      <c r="AU7" t="n">
+        <v>75472</v>
+      </c>
+      <c r="AV7" t="n">
+        <v>75136</v>
+      </c>
+      <c r="AW7" t="n">
+        <v>78149</v>
+      </c>
+      <c r="AX7" t="n">
         <v>76095</v>
       </c>
-      <c r="C7" t="n">
+      <c r="AY7" t="n">
         <v>74519</v>
       </c>
-      <c r="D7" t="n">
+      <c r="AZ7" t="n">
         <v>75387</v>
       </c>
-      <c r="E7" t="n">
+      <c r="BA7" t="n">
         <v>78056</v>
       </c>
-      <c r="F7" t="n">
+      <c r="BB7" t="n">
         <v>80218</v>
       </c>
-      <c r="G7" t="n">
+      <c r="BC7" t="n">
         <v>79017</v>
       </c>
-      <c r="H7" t="n">
+      <c r="BD7" t="n">
         <v>79458</v>
       </c>
-      <c r="I7" t="n">
+      <c r="BE7" t="n">
         <v>80964</v>
       </c>
-      <c r="J7" t="n">
+      <c r="BF7" t="n">
         <v>76411</v>
       </c>
-      <c r="K7" t="n">
+      <c r="BG7" t="n">
         <v>77353</v>
       </c>
-      <c r="L7" t="n">
+      <c r="BH7" t="n">
         <v>79282</v>
       </c>
-      <c r="M7" t="n">
+      <c r="BI7" t="n">
         <v>79729</v>
       </c>
-      <c r="N7" t="n">
+      <c r="BJ7" t="n">
         <v>82059</v>
       </c>
-      <c r="O7" t="n">
+      <c r="BK7" t="n">
         <v>80984</v>
       </c>
-      <c r="P7" t="n">
+      <c r="BL7" t="n">
         <v>81835</v>
       </c>
-      <c r="Q7" t="n">
+      <c r="BM7" t="n">
         <v>86299</v>
       </c>
-      <c r="R7" t="n">
+      <c r="BN7" t="n">
         <v>86006</v>
       </c>
-      <c r="S7" t="n">
+      <c r="BO7" t="n">
         <v>86474</v>
       </c>
-      <c r="T7" t="n">
+      <c r="BP7" t="n">
         <v>86488</v>
       </c>
-      <c r="U7" t="n">
+      <c r="BQ7" t="n">
         <v>86550</v>
       </c>
-      <c r="V7" t="n">
+      <c r="BR7" t="n">
         <v>84626</v>
       </c>
-      <c r="W7" t="n">
+      <c r="BS7" t="n">
         <v>85070</v>
       </c>
-      <c r="X7" t="n">
+      <c r="BT7" t="n">
         <v>87525</v>
       </c>
-      <c r="Y7" t="n">
+      <c r="BU7" t="n">
         <v>89914</v>
       </c>
-      <c r="Z7" t="n">
+      <c r="BV7" t="n">
         <v>88305</v>
       </c>
-      <c r="AA7" t="n">
+      <c r="BW7" t="n">
         <v>88288</v>
       </c>
-      <c r="AB7" t="n">
+      <c r="BX7" t="n">
         <v>89875</v>
       </c>
-      <c r="AC7" t="n">
+      <c r="BY7" t="n">
         <v>93627</v>
       </c>
-      <c r="AD7" t="n">
+      <c r="BZ7" t="n">
         <v>95171</v>
       </c>
-      <c r="AE7" t="n">
+      <c r="CA7" t="n">
         <v>94963</v>
       </c>
-      <c r="AF7" t="n">
+      <c r="CB7" t="n">
         <v>95929</v>
       </c>
-      <c r="AG7" t="n">
+      <c r="CC7" t="n">
         <v>97153</v>
       </c>
-      <c r="AH7" t="n">
+      <c r="CD7" t="n">
         <v>99088</v>
       </c>
-      <c r="AI7" t="n">
+      <c r="CE7" t="n">
         <v>94663</v>
       </c>
-      <c r="AJ7" t="n">
+      <c r="CF7" t="n">
         <v>94505</v>
       </c>
-      <c r="AK7" t="n">
+      <c r="CG7" t="n">
         <v>93879</v>
       </c>
-      <c r="AL7" t="n">
+      <c r="CH7" t="n">
         <v>90209</v>
       </c>
-      <c r="AM7" t="n">
+      <c r="CI7" t="n">
         <v>91801</v>
       </c>
-      <c r="AN7" t="n">
+      <c r="CJ7" t="n">
         <v>97780</v>
       </c>
-      <c r="AO7" t="n">
+      <c r="CK7" t="n">
         <v>95814</v>
       </c>
-      <c r="AP7" t="n">
+      <c r="CL7" t="n">
         <v>96089</v>
       </c>
-      <c r="AQ7" t="n">
+      <c r="CM7" t="n">
         <v>98529</v>
       </c>
-      <c r="AR7" t="n">
+      <c r="CN7" t="n">
         <v>97607</v>
       </c>
-      <c r="AS7" t="n">
+      <c r="CO7" t="n">
         <v>98412</v>
       </c>
-      <c r="AT7" t="n">
+      <c r="CP7" t="n">
         <v>97141</v>
       </c>
-      <c r="AU7" t="n">
+      <c r="CQ7" t="n">
         <v>99676</v>
       </c>
-      <c r="AV7" t="n">
+      <c r="CR7" t="n">
         <v>98608</v>
       </c>
-      <c r="AW7" t="n">
+      <c r="CS7" t="n">
         <v>98396</v>
       </c>
-      <c r="AX7" t="n">
+      <c r="CT7" t="n">
         <v>98880</v>
       </c>
-      <c r="AY7" t="n">
+      <c r="CU7" t="n">
         <v>98078</v>
       </c>
-      <c r="AZ7" t="n">
+      <c r="CV7" t="n">
         <v>97132</v>
       </c>
-      <c r="BA7" t="n">
+      <c r="CW7" t="n">
         <v>96496</v>
       </c>
-      <c r="BB7" t="n">
+      <c r="CX7" t="n">
         <v>96721</v>
       </c>
-      <c r="BC7" t="n">
+      <c r="CY7" t="n">
         <v>96543</v>
       </c>
-      <c r="BD7" t="n">
+      <c r="CZ7" t="n">
         <v>96979</v>
       </c>
-      <c r="BE7" t="n">
+      <c r="DA7" t="n">
         <v>97109</v>
       </c>
     </row>
@@ -3566,170 +4677,315 @@
         </is>
       </c>
       <c r="B8" t="n">
+        <v>785721</v>
+      </c>
+      <c r="C8" t="n">
+        <v>775859.48</v>
+      </c>
+      <c r="D8" t="n">
+        <v>772163.11</v>
+      </c>
+      <c r="E8" t="n">
+        <v>763450.66</v>
+      </c>
+      <c r="F8" t="n">
+        <v>751320.5600000001</v>
+      </c>
+      <c r="G8" t="n">
+        <v>753024.61</v>
+      </c>
+      <c r="H8" t="n">
+        <v>757826.1800000001</v>
+      </c>
+      <c r="I8" t="n">
+        <v>754357.7</v>
+      </c>
+      <c r="J8" t="n">
+        <v>757259.58</v>
+      </c>
+      <c r="K8" t="n">
+        <v>748291.83</v>
+      </c>
+      <c r="L8" t="n">
+        <v>749667.66</v>
+      </c>
+      <c r="M8" t="n">
+        <v>738430.58</v>
+      </c>
+      <c r="N8" t="n">
+        <v>746148.9399999999</v>
+      </c>
+      <c r="O8" t="n">
+        <v>741494.59</v>
+      </c>
+      <c r="P8" t="n">
+        <v>759836.37</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>758102.87</v>
+      </c>
+      <c r="R8" t="n">
+        <v>755227.49</v>
+      </c>
+      <c r="S8" t="n">
+        <v>778290.28</v>
+      </c>
+      <c r="T8" t="n">
+        <v>775108.41</v>
+      </c>
+      <c r="U8" t="n">
+        <v>776404.39</v>
+      </c>
+      <c r="V8" t="n">
+        <v>779738.05</v>
+      </c>
+      <c r="W8" t="n">
+        <v>789596.8100000001</v>
+      </c>
+      <c r="X8" t="n">
+        <v>782186.6899999999</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>798088.9300000001</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>791220.73</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>795067.9300000001</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>791209.92</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>824698.24</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>847790.79</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>896142.1899999999</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>929363.02</v>
+      </c>
+      <c r="AG8" t="n">
+        <v>940000.97</v>
+      </c>
+      <c r="AH8" t="n">
+        <v>945482.64</v>
+      </c>
+      <c r="AI8" t="n">
+        <v>952031.8</v>
+      </c>
+      <c r="AJ8" t="n">
+        <v>970217.97</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>1013189.38</v>
+      </c>
+      <c r="AL8" t="n">
+        <v>1009454.8</v>
+      </c>
+      <c r="AM8" t="n">
+        <v>1009526.08</v>
+      </c>
+      <c r="AN8" t="n">
+        <v>988393.95</v>
+      </c>
+      <c r="AO8" t="n">
+        <v>1004279.84</v>
+      </c>
+      <c r="AP8" t="n">
+        <v>1002450.44</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>1018809.18</v>
+      </c>
+      <c r="AR8" t="n">
+        <v>1018181.25</v>
+      </c>
+      <c r="AS8" t="n">
+        <v>1018628</v>
+      </c>
+      <c r="AT8" t="n">
+        <v>1004402.44</v>
+      </c>
+      <c r="AU8" t="n">
+        <v>1011822.22</v>
+      </c>
+      <c r="AV8" t="n">
+        <v>1005964.72</v>
+      </c>
+      <c r="AW8" t="n">
+        <v>1033798.65</v>
+      </c>
+      <c r="AX8" t="n">
         <v>1017415.33</v>
       </c>
-      <c r="C8" t="n">
+      <c r="AY8" t="n">
         <v>1021205.09</v>
       </c>
-      <c r="D8" t="n">
+      <c r="AZ8" t="n">
         <v>985078.61</v>
       </c>
-      <c r="E8" t="n">
+      <c r="BA8" t="n">
         <v>953465.0699999999</v>
       </c>
-      <c r="F8" t="n">
+      <c r="BB8" t="n">
         <v>964651.0600000001</v>
       </c>
-      <c r="G8" t="n">
+      <c r="BC8" t="n">
         <v>887448.48</v>
       </c>
-      <c r="H8" t="n">
+      <c r="BD8" t="n">
         <v>887071.83</v>
       </c>
-      <c r="I8" t="n">
+      <c r="BE8" t="n">
         <v>877562.25</v>
       </c>
-      <c r="J8" t="n">
+      <c r="BF8" t="n">
         <v>822339.5</v>
       </c>
-      <c r="K8" t="n">
+      <c r="BG8" t="n">
         <v>814555.6899999999</v>
       </c>
-      <c r="L8" t="n">
+      <c r="BH8" t="n">
         <v>832856.42</v>
       </c>
-      <c r="M8" t="n">
+      <c r="BI8" t="n">
         <v>848509.64</v>
       </c>
-      <c r="N8" t="n">
+      <c r="BJ8" t="n">
         <v>850924.63</v>
       </c>
-      <c r="O8" t="n">
+      <c r="BK8" t="n">
         <v>822856.41</v>
       </c>
-      <c r="P8" t="n">
+      <c r="BL8" t="n">
         <v>813080.99</v>
       </c>
-      <c r="Q8" t="n">
+      <c r="BM8" t="n">
         <v>819722.55</v>
       </c>
-      <c r="R8" t="n">
+      <c r="BN8" t="n">
         <v>805716.7</v>
       </c>
-      <c r="S8" t="n">
+      <c r="BO8" t="n">
         <v>808190.39</v>
       </c>
-      <c r="T8" t="n">
+      <c r="BP8" t="n">
         <v>803228.9</v>
       </c>
-      <c r="U8" t="n">
+      <c r="BQ8" t="n">
         <v>785734.47</v>
       </c>
-      <c r="V8" t="n">
+      <c r="BR8" t="n">
         <v>741365.63</v>
       </c>
-      <c r="W8" t="n">
+      <c r="BS8" t="n">
         <v>724518.23</v>
       </c>
-      <c r="X8" t="n">
+      <c r="BT8" t="n">
         <v>733629.27</v>
       </c>
-      <c r="Y8" t="n">
+      <c r="BU8" t="n">
         <v>779970.87</v>
       </c>
-      <c r="Z8" t="n">
+      <c r="BV8" t="n">
         <v>773682.26</v>
       </c>
-      <c r="AA8" t="n">
+      <c r="BW8" t="n">
         <v>771212.3100000001</v>
       </c>
-      <c r="AB8" t="n">
+      <c r="BX8" t="n">
         <v>793167.83</v>
       </c>
-      <c r="AC8" t="n">
+      <c r="BY8" t="n">
         <v>787294.66</v>
       </c>
-      <c r="AD8" t="n">
+      <c r="BZ8" t="n">
         <v>795406.01</v>
       </c>
-      <c r="AE8" t="n">
+      <c r="CA8" t="n">
         <v>791623.08</v>
       </c>
-      <c r="AF8" t="n">
+      <c r="CB8" t="n">
         <v>801978.47</v>
       </c>
-      <c r="AG8" t="n">
+      <c r="CC8" t="n">
         <v>816745.33</v>
       </c>
-      <c r="AH8" t="n">
+      <c r="CD8" t="n">
         <v>847502.5</v>
       </c>
-      <c r="AI8" t="n">
+      <c r="CE8" t="n">
         <v>831453.6800000001</v>
       </c>
-      <c r="AJ8" t="n">
+      <c r="CF8" t="n">
         <v>822005.26</v>
       </c>
-      <c r="AK8" t="n">
+      <c r="CG8" t="n">
         <v>808024.55</v>
       </c>
-      <c r="AL8" t="n">
+      <c r="CH8" t="n">
         <v>809259.3100000001</v>
       </c>
-      <c r="AM8" t="n">
+      <c r="CI8" t="n">
         <v>814973.0600000001</v>
       </c>
-      <c r="AN8" t="n">
+      <c r="CJ8" t="n">
         <v>822339.5</v>
       </c>
-      <c r="AO8" t="n">
+      <c r="CK8" t="n">
         <v>854313.96</v>
       </c>
-      <c r="AP8" t="n">
+      <c r="CL8" t="n">
         <v>854058.97</v>
       </c>
-      <c r="AQ8" t="n">
+      <c r="CM8" t="n">
         <v>894234.6</v>
       </c>
-      <c r="AR8" t="n">
+      <c r="CN8" t="n">
         <v>880000.59</v>
       </c>
-      <c r="AS8" t="n">
+      <c r="CO8" t="n">
         <v>892783.55</v>
       </c>
-      <c r="AT8" t="n">
+      <c r="CP8" t="n">
         <v>911657.16</v>
       </c>
-      <c r="AU8" t="n">
+      <c r="CQ8" t="n">
         <v>902110.0699999999</v>
       </c>
-      <c r="AV8" t="n">
+      <c r="CR8" t="n">
         <v>903578.55</v>
       </c>
-      <c r="AW8" t="n">
+      <c r="CS8" t="n">
         <v>914657.72</v>
       </c>
-      <c r="AX8" t="n">
+      <c r="CT8" t="n">
         <v>926074.95</v>
       </c>
-      <c r="AY8" t="n">
+      <c r="CU8" t="n">
         <v>923641.88</v>
       </c>
-      <c r="AZ8" t="n">
+      <c r="CV8" t="n">
         <v>901037.53</v>
       </c>
-      <c r="BA8" t="n">
+      <c r="CW8" t="n">
         <v>912992.02</v>
       </c>
-      <c r="BB8" t="n">
+      <c r="CX8" t="n">
         <v>909891.41</v>
       </c>
-      <c r="BC8" t="n">
+      <c r="CY8" t="n">
         <v>938059.96</v>
       </c>
-      <c r="BD8" t="n">
+      <c r="CZ8" t="n">
         <v>945802.5699999999</v>
       </c>
+      <c r="DA8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3738,171 +4994,315 @@
         </is>
       </c>
       <c r="B9" t="n">
+        <v>20112</v>
+      </c>
+      <c r="C9" t="n">
+        <v>19346</v>
+      </c>
+      <c r="D9" t="n">
+        <v>20331</v>
+      </c>
+      <c r="E9" t="n">
+        <v>19268</v>
+      </c>
+      <c r="F9" t="n">
+        <v>20082</v>
+      </c>
+      <c r="G9" t="n">
+        <v>20353</v>
+      </c>
+      <c r="H9" t="n">
+        <v>18724</v>
+      </c>
+      <c r="I9" t="n">
+        <v>19272</v>
+      </c>
+      <c r="J9" t="n">
+        <v>18629</v>
+      </c>
+      <c r="K9" t="n">
+        <v>16499</v>
+      </c>
+      <c r="L9" t="n">
+        <v>16514</v>
+      </c>
+      <c r="M9" t="n">
+        <v>16060</v>
+      </c>
+      <c r="N9" t="n">
+        <v>18782</v>
+      </c>
+      <c r="O9" t="n">
+        <v>18085</v>
+      </c>
+      <c r="P9" t="n">
+        <v>17301</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>16586</v>
+      </c>
+      <c r="R9" t="n">
+        <v>17536</v>
+      </c>
+      <c r="S9" t="n">
+        <v>18039</v>
+      </c>
+      <c r="T9" t="n">
+        <v>16196</v>
+      </c>
+      <c r="U9" t="n">
+        <v>15827</v>
+      </c>
+      <c r="V9" t="n">
+        <v>16849</v>
+      </c>
+      <c r="W9" t="n">
+        <v>16012</v>
+      </c>
+      <c r="X9" t="n">
+        <v>16804</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>16264</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>17958</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>18070</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>21964</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>18806</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>17764</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>19547</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>17506</v>
+      </c>
+      <c r="AG9" t="n">
+        <v>14771</v>
+      </c>
+      <c r="AH9" t="n">
+        <v>12612</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>11621</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>12263</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>12005</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>11686</v>
+      </c>
+      <c r="AM9" t="n">
+        <v>11542</v>
+      </c>
+      <c r="AN9" t="n">
+        <v>11228</v>
+      </c>
+      <c r="AO9" t="n">
+        <v>12865</v>
+      </c>
+      <c r="AP9" t="n">
+        <v>11880</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>12251</v>
+      </c>
+      <c r="AR9" t="n">
+        <v>10590</v>
+      </c>
+      <c r="AS9" t="n">
+        <v>12478</v>
+      </c>
+      <c r="AT9" t="n">
+        <v>12110</v>
+      </c>
+      <c r="AU9" t="n">
+        <v>13349</v>
+      </c>
+      <c r="AV9" t="n">
+        <v>11438</v>
+      </c>
+      <c r="AW9" t="n">
+        <v>12665</v>
+      </c>
+      <c r="AX9" t="n">
         <v>11132</v>
       </c>
-      <c r="C9" t="n">
+      <c r="AY9" t="n">
         <v>11012</v>
       </c>
-      <c r="D9" t="n">
+      <c r="AZ9" t="n">
         <v>12794</v>
       </c>
-      <c r="E9" t="n">
+      <c r="BA9" t="n">
         <v>8547</v>
       </c>
-      <c r="F9" t="n">
+      <c r="BB9" t="n">
         <v>11076</v>
       </c>
-      <c r="G9" t="n">
+      <c r="BC9" t="n">
         <v>9127</v>
       </c>
-      <c r="H9" t="n">
+      <c r="BD9" t="n">
         <v>10034</v>
       </c>
-      <c r="I9" t="n">
+      <c r="BE9" t="n">
         <v>8685</v>
       </c>
-      <c r="J9" t="n">
+      <c r="BF9" t="n">
         <v>8231</v>
       </c>
-      <c r="K9" t="n">
+      <c r="BG9" t="n">
         <v>6716</v>
       </c>
-      <c r="L9" t="n">
+      <c r="BH9" t="n">
         <v>11377</v>
       </c>
-      <c r="M9" t="n">
+      <c r="BI9" t="n">
         <v>11061</v>
       </c>
-      <c r="N9" t="n">
+      <c r="BJ9" t="n">
         <v>11419</v>
       </c>
-      <c r="O9" t="n">
+      <c r="BK9" t="n">
         <v>13462</v>
       </c>
-      <c r="P9" t="n">
+      <c r="BL9" t="n">
         <v>11364</v>
       </c>
-      <c r="Q9" t="n">
+      <c r="BM9" t="n">
         <v>12534</v>
       </c>
-      <c r="R9" t="n">
+      <c r="BN9" t="n">
         <v>12544</v>
       </c>
-      <c r="S9" t="n">
+      <c r="BO9" t="n">
         <v>9934</v>
       </c>
-      <c r="T9" t="n">
+      <c r="BP9" t="n">
         <v>13615</v>
       </c>
-      <c r="U9" t="n">
+      <c r="BQ9" t="n">
         <v>12940</v>
       </c>
-      <c r="V9" t="n">
+      <c r="BR9" t="n">
         <v>13708</v>
       </c>
-      <c r="W9" t="n">
+      <c r="BS9" t="n">
         <v>12577</v>
       </c>
-      <c r="X9" t="n">
+      <c r="BT9" t="n">
         <v>15987</v>
       </c>
-      <c r="Y9" t="n">
+      <c r="BU9" t="n">
         <v>12113</v>
       </c>
-      <c r="Z9" t="n">
+      <c r="BV9" t="n">
         <v>14893</v>
       </c>
-      <c r="AA9" t="n">
+      <c r="BW9" t="n">
         <v>15975</v>
       </c>
-      <c r="AB9" t="n">
+      <c r="BX9" t="n">
         <v>12891</v>
       </c>
-      <c r="AC9" t="n">
+      <c r="BY9" t="n">
         <v>15712</v>
       </c>
-      <c r="AD9" t="n">
+      <c r="BZ9" t="n">
         <v>14660</v>
       </c>
-      <c r="AE9" t="n">
+      <c r="CA9" t="n">
         <v>14485</v>
       </c>
-      <c r="AF9" t="n">
+      <c r="CB9" t="n">
         <v>17689</v>
       </c>
-      <c r="AG9" t="n">
+      <c r="CC9" t="n">
         <v>17055</v>
       </c>
-      <c r="AH9" t="n">
+      <c r="CD9" t="n">
         <v>17316</v>
       </c>
-      <c r="AI9" t="n">
+      <c r="CE9" t="n">
         <v>20275</v>
       </c>
-      <c r="AJ9" t="n">
+      <c r="CF9" t="n">
         <v>19174</v>
       </c>
-      <c r="AK9" t="n">
+      <c r="CG9" t="n">
         <v>18836</v>
       </c>
-      <c r="AL9" t="n">
+      <c r="CH9" t="n">
         <v>23379</v>
       </c>
-      <c r="AM9" t="n">
+      <c r="CI9" t="n">
         <v>24951</v>
       </c>
-      <c r="AN9" t="n">
+      <c r="CJ9" t="n">
         <v>22603</v>
       </c>
-      <c r="AO9" t="n">
+      <c r="CK9" t="n">
         <v>23387</v>
       </c>
-      <c r="AP9" t="n">
+      <c r="CL9" t="n">
         <v>24600</v>
       </c>
-      <c r="AQ9" t="n">
+      <c r="CM9" t="n">
         <v>24320</v>
       </c>
-      <c r="AR9" t="n">
+      <c r="CN9" t="n">
         <v>25170</v>
       </c>
-      <c r="AS9" t="n">
+      <c r="CO9" t="n">
         <v>24884</v>
       </c>
-      <c r="AT9" t="n">
+      <c r="CP9" t="n">
         <v>24006</v>
       </c>
-      <c r="AU9" t="n">
+      <c r="CQ9" t="n">
         <v>24202</v>
       </c>
-      <c r="AV9" t="n">
+      <c r="CR9" t="n">
         <v>28622</v>
       </c>
-      <c r="AW9" t="n">
+      <c r="CS9" t="n">
         <v>24781</v>
       </c>
-      <c r="AX9" t="n">
+      <c r="CT9" t="n">
         <v>27582</v>
       </c>
-      <c r="AY9" t="n">
+      <c r="CU9" t="n">
         <v>25799</v>
       </c>
-      <c r="AZ9" t="n">
+      <c r="CV9" t="n">
         <v>31400</v>
       </c>
-      <c r="BA9" t="n">
+      <c r="CW9" t="n">
         <v>27963</v>
       </c>
-      <c r="BB9" t="n">
+      <c r="CX9" t="n">
         <v>29170</v>
       </c>
-      <c r="BC9" t="n">
+      <c r="CY9" t="n">
         <v>26032</v>
       </c>
-      <c r="BD9" t="n">
+      <c r="CZ9" t="n">
         <v>26599</v>
       </c>
-      <c r="BE9" t="n">
+      <c r="DA9" t="n">
         <v>25646</v>
       </c>
     </row>

</xml_diff>